<commit_message>
OK for the output style
</commit_message>
<xml_diff>
--- a/rag/excel/baseline_vs_rag.xlsx
+++ b/rag/excel/baseline_vs_rag.xlsx
@@ -776,7 +776,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MonCal.Facts.RF</t>
+          <t>MonCal.Interpret</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>MonCal.Facts.DC</t>
+          <t>MonCal.Facts.RF</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>MonCal.Facts.DC</t>
+          <t>MonCal.Facts.RF</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>MonCal.Facts.RF</t>
+          <t>MonCal.Facts.DC</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>MonCal.Facts.RF</t>
+          <t>MonCal.Facts.DC</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2116,17 +2116,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Question après question, j’étais plutôt sûre de moi.</t>
+          <t>Globalement, il y a beaucoup de réponses correctes, (17 sur 24)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>MonCal.Facts.DC</t>
+          <t>MonCal.Facts.RF</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>MonCal.Facts.DC</t>
+          <t>MotOrient.SelfEff</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2211,12 +2211,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>MonCal.Facts.RF</t>
+          <t>MonCal.Facts.DC</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>MonCal.Facts.RF</t>
+          <t>MonCal.Facts.DC</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>MonCal.Facts.RF</t>
+          <t>MonCal.Facts.DC</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>MotOrient.SelfEff</t>
+          <t>MonCal.Facts.DC</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -3351,7 +3351,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>MonCal.Facts.DC</t>
+          <t>MonCal.Facts.RF</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>MonCal.Facts.DC</t>
+          <t>MotOrient.SelfEff</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>StratKldg</t>
+          <t>CTRL</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>MonCal.Facts.RF</t>
+          <t>MonCal.Facts.DC</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -4461,7 +4461,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>MonCal.Facts.RF</t>
+          <t>MonCal.Facts.DC</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -4796,7 +4796,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>MonCal.Facts.DC</t>
+          <t>MonCal.Facts.RF</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>CTRL</t>
+          <t>DomKldg</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -5276,7 +5276,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>DomKldg</t>
+          <t>MonCal.Facts.DC</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -5296,17 +5296,17 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Ce score global montre des connaissances mais quelques partialités en général.</t>
+          <t>Les erreurs dangereuses en était globalement peut nombreuse mêmes si ce n’est pas encore ça, mais je trouve que j’ai un savoir un peu fragile même si globalement c’est bien.</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>DomKldg</t>
+          <t>MonCal.Interpret</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>StratKldg</t>
+          <t>MonCal.Facts.DC</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>MonCal.Facts.DC</t>
+          <t>MonCal.Facts.RF</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
@@ -6076,7 +6076,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Globalement, mon score est correct (équivaut à 16/20)</t>
+          <t>Mon résultat 30/40 , 8 réponses incorrectes , 5 ignorances , 27 réponses correctes</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -6111,12 +6111,12 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>MonCal.Facts.DC</t>
+          <t>MonCal.Facts.RF</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>StratKldg</t>
+          <t>MonCal.Facts.DC</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -7276,12 +7276,12 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>plusieurs mauvaises réponses dues à un oubli de cours</t>
+          <t>on peut penser que je suis assez prudent</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>DomKldg</t>
+          <t>MonCal.Interpret</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">

</xml_diff>